<commit_message>
Todos los documentos listos y subidos
</commit_message>
<xml_diff>
--- a/FINAL FASE 1/Anexos/Gestión/Carta Gantt.xlsx
+++ b/FINAL FASE 1/Anexos/Gestión/Carta Gantt.xlsx
@@ -2085,13 +2085,13 @@
     <row r="1001" ht="14.25" customHeight="1"/>
   </sheetData>
   <mergeCells count="7">
+    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="A2:T2"/>
     <mergeCell ref="A4:A6"/>
     <mergeCell ref="B4:E4"/>
     <mergeCell ref="F4:P4"/>
+    <mergeCell ref="Q4:R4"/>
     <mergeCell ref="A30:J30"/>
-    <mergeCell ref="A1:T1"/>
-    <mergeCell ref="A2:T2"/>
-    <mergeCell ref="Q4:R4"/>
   </mergeCells>
   <printOptions/>
   <pageMargins bottom="0.4" footer="0.0" header="0.0" left="0.3" right="0.3" top="0.4"/>

</xml_diff>